<commit_message>
cart scenarios for one/multiple items done
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\Python\QA_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{0336A98B-5E7C-42C2-B3A3-15D52BD87D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55028694-0C0A-4159-8D21-2258E63EC8C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8FBF4EF6-23A4-453E-A09F-460DDE2B30EF}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,22 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
-  <si>
-    <t>Given</t>
-  </si>
-  <si>
-    <t>When</t>
-  </si>
-  <si>
-    <t>Then</t>
-  </si>
-  <si>
-    <t>user enters valid register details</t>
-  </si>
-  <si>
-    <t>user is on register page</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
   <si>
     <t>ID</t>
   </si>
@@ -69,22 +53,10 @@
     <t>Priority</t>
   </si>
   <si>
-    <t>user is logged in</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
-    <t>user enters invalid register details</t>
-  </si>
-  <si>
-    <t>user gets specific error</t>
-  </si>
-  <si>
-    <t>user is on login page</t>
-  </si>
-  <si>
-    <t>user enters valid login details</t>
+    <t>OCD_Register_003</t>
   </si>
   <si>
     <t>OCD_Login_002</t>
@@ -93,54 +65,21 @@
     <t>OCD_Login_001</t>
   </si>
   <si>
-    <t>user enters invalid login details</t>
-  </si>
-  <si>
-    <t>user gets login error</t>
-  </si>
-  <si>
     <t>OCD_Search_001</t>
   </si>
   <si>
-    <t>user is on home page</t>
-  </si>
-  <si>
-    <t>user can see the product</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
-    <t>user searches for valid product and presses 'enter'</t>
-  </si>
-  <si>
     <t>OCD_Search_002</t>
   </si>
   <si>
-    <t>user searches for valid product and presses 'Search' button</t>
-  </si>
-  <si>
     <t>OCD_Search_003</t>
   </si>
   <si>
-    <t>user searches for invalid product and presses 'Search' button</t>
-  </si>
-  <si>
-    <t>user can see page with no results</t>
-  </si>
-  <si>
     <t>OCD_Cart_001</t>
   </si>
   <si>
-    <t>user is on product page</t>
-  </si>
-  <si>
-    <t>user presses 'add to cart' on product</t>
-  </si>
-  <si>
-    <t>user can see product in cart</t>
-  </si>
-  <si>
     <t>OCD_Cart_002</t>
   </si>
   <si>
@@ -150,15 +89,9 @@
     <t>user can see total cost of cart items</t>
   </si>
   <si>
-    <t xml:space="preserve"> user is on product page</t>
-  </si>
-  <si>
     <t>OCD_Cart_003</t>
   </si>
   <si>
-    <t>user in on home page</t>
-  </si>
-  <si>
     <t>user removes item from cart</t>
   </si>
   <si>
@@ -166,6 +99,220 @@
   </si>
   <si>
     <t>Critical</t>
+  </si>
+  <si>
+    <t>Preconditions</t>
+  </si>
+  <si>
+    <t>Expected Results</t>
+  </si>
+  <si>
+    <t>Step-by-Step Instructions</t>
+  </si>
+  <si>
+    <t>Clean browser instance
+Internet connection
+The email is not already used
+User is on the register page</t>
+  </si>
+  <si>
+    <t>Clean browser instance
+Internet connection
+User is on the register page</t>
+  </si>
+  <si>
+    <t>Internet connection
+Clean browser instance
+User is on login page</t>
+  </si>
+  <si>
+    <t>Internet connection
+Clean browser instance
+Current account was registered
+User is on login page</t>
+  </si>
+  <si>
+    <t>OCD_Login_003</t>
+  </si>
+  <si>
+    <t>Internet connection
+Clean browser instance
+User is on home page</t>
+  </si>
+  <si>
+    <t>Internet connection
+Clean browser instance
+User is on any page</t>
+  </si>
+  <si>
+    <t>Internet connection
+Clean browser instance
+User in on any page</t>
+  </si>
+  <si>
+    <t>1. user enters first name, last name, email, phone number, password, confirmed password
+2. checks subscription box
+3. checks privacy acceptance box
+4. Clicks 'Continue' button</t>
+  </si>
+  <si>
+    <t>OCD_Nav_001</t>
+  </si>
+  <si>
+    <t>User is on the home page</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Successful registration</t>
+  </si>
+  <si>
+    <t>Successful login</t>
+  </si>
+  <si>
+    <t>Wrong password on login</t>
+  </si>
+  <si>
+    <t>Invalid credentials on login</t>
+  </si>
+  <si>
+    <t>Product search with 'enter'</t>
+  </si>
+  <si>
+    <t>Product search with Button</t>
+  </si>
+  <si>
+    <t>Invalid product search</t>
+  </si>
+  <si>
+    <t>Adding to cart successful</t>
+  </si>
+  <si>
+    <t>Multiple products added
+added to cart</t>
+  </si>
+  <si>
+    <t>Product removal from cart</t>
+  </si>
+  <si>
+    <t>1. user enters first name, last name, email, phone number, password, confirmed password
+2. checks subscription box
+4. Clicks 'Continue' button</t>
+  </si>
+  <si>
+    <t>Failed registration due to
+policy not being accepted</t>
+  </si>
+  <si>
+    <t>Failed registration due to wrong password confirm-
+ation</t>
+  </si>
+  <si>
+    <t>1. user enters first name, last name, email, phone number, password, wrong confirmed password
+2. checks subscription box
+3. checks privacy acceptance box
+4. Clicks 'Continue' button</t>
+  </si>
+  <si>
+    <t>Registration error should not be visible
+User gets redirected to Registration Success page</t>
+  </si>
+  <si>
+    <t>Registration error appears: Warning: 'You must agree to the 
+Privacy Policy!'</t>
+  </si>
+  <si>
+    <t>Registration error appears: Password confirmation does not match password!</t>
+  </si>
+  <si>
+    <t>Navigation from home -&gt; 
+registration</t>
+  </si>
+  <si>
+    <t>OCD_Nav_002</t>
+  </si>
+  <si>
+    <t>Navigation from home -&gt; login</t>
+  </si>
+  <si>
+    <t>1. Click account logo
+2. Click 'Login' button in popup</t>
+  </si>
+  <si>
+    <t>1. Click account logo
+2. Click 'Register' button in popup</t>
+  </si>
+  <si>
+    <t>user gets to login page</t>
+  </si>
+  <si>
+    <t>user gets to register page</t>
+  </si>
+  <si>
+    <t>user gets to account page</t>
+  </si>
+  <si>
+    <t>user should see error "Warning: No match for E-Mail Address and/or 
+Password."</t>
+  </si>
+  <si>
+    <t>1. user enters correct email in the 'email' field
+2. user enters correct password in the 'password' field
+3. clicks the 'Login' button</t>
+  </si>
+  <si>
+    <t>1. user enters invalid email in the 'email' field
+2. user enters invalid password in the 'password' field
+3. user clicks 'Login' button</t>
+  </si>
+  <si>
+    <t>1. user enters valid email in the 'email' field
+2. user enters wrong password in the 'password' field
+3. user clicks 'Login' button</t>
+  </si>
+  <si>
+    <t>OCD_Login_004</t>
+  </si>
+  <si>
+    <t>SQL Injection attempt on 
+password field</t>
+  </si>
+  <si>
+    <t>1. user enters valid email in the 'email' field
+2. user enters sql injection line &lt;password' or 1=1;--&gt; in the 'password' field
+3. user clicks 'Login' button</t>
+  </si>
+  <si>
+    <t>Internet connection
+Clean browser instance
+User is on any page
+4 'Mac' products are present in the db</t>
+  </si>
+  <si>
+    <t>1. user enters "Mac" in the search bar on top
+2. clicks the 'Search' button</t>
+  </si>
+  <si>
+    <t>User should see 4 products: iMac, MacBook, MacBook Air, MacBook Pro</t>
+  </si>
+  <si>
+    <t>1. user enters "Mac" in the search bar on top
+2. taps Enter key on keyboard</t>
+  </si>
+  <si>
+    <t>1. user enters "magic tree" in the search bar on top
+2. clicks the 'Search' button</t>
+  </si>
+  <si>
+    <t>user can see: "There is no product that matches the search criteria."</t>
+  </si>
+  <si>
+    <t>1. user scrolls to the first product on home page
+2. clicks the 'Add to Cart' button</t>
+  </si>
+  <si>
+    <t>cart status should update on the right-top side</t>
   </si>
 </sst>
 </file>
@@ -201,8 +348,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,200 +687,334 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A021F8-77F7-49B4-AF4C-68F5356311C2}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="52.140625" customWidth="1"/>
-    <col min="3" max="3" width="68" customWidth="1"/>
-    <col min="4" max="4" width="62.7109375" customWidth="1"/>
+    <col min="1" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="52.140625" customWidth="1"/>
+    <col min="4" max="4" width="68" customWidth="1"/>
+    <col min="5" max="5" width="64.5703125" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+    </row>
+    <row r="10" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>32</v>
       </c>
-      <c r="E9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" t="s">
-        <v>22</v>
+      <c r="D15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cart scenarios improved and more generic functions
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\Python\QA_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55028694-0C0A-4159-8D21-2258E63EC8C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5738143-B461-46C0-9DC0-A38418DF91B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8FBF4EF6-23A4-453E-A09F-460DDE2B30EF}"/>
   </bookViews>
@@ -83,19 +83,7 @@
     <t>OCD_Cart_002</t>
   </si>
   <si>
-    <t>user adds more products to cart</t>
-  </si>
-  <si>
-    <t>user can see total cost of cart items</t>
-  </si>
-  <si>
     <t>OCD_Cart_003</t>
-  </si>
-  <si>
-    <t>user removes item from cart</t>
-  </si>
-  <si>
-    <t>user can see 1 less item in cart</t>
   </si>
   <si>
     <t>Critical</t>
@@ -145,11 +133,6 @@
 User is on any page</t>
   </si>
   <si>
-    <t>Internet connection
-Clean browser instance
-User in on any page</t>
-  </si>
-  <si>
     <t>1. user enters first name, last name, email, phone number, password, confirmed password
 2. checks subscription box
 3. checks privacy acceptance box
@@ -313,6 +296,29 @@
   </si>
   <si>
     <t>cart status should update on the right-top side</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. user enters "mac" and presses 'Enter' in the search bar
+2. adds "iMac" to cart
+3. adds "MacBook Air" to cart
+</t>
+  </si>
+  <si>
+    <t>user should see cart status "2 item(s) - $1,324.00"</t>
+  </si>
+  <si>
+    <t>Internet connection
+Clean browser instance
+User in on home page</t>
+  </si>
+  <si>
+    <t>1. user enters "samsung" and presses 'Enter' in the search bar
+2. adds product "Samsung SyncMaster 941BW" to cart
+4. clicks cart icon
+3. deletes "Samsung SyncMaster 941BW" from cart</t>
+  </si>
+  <si>
+    <t>user can see empty cart</t>
   </si>
 </sst>
 </file>
@@ -702,16 +708,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -722,16 +728,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
         <v>4</v>
@@ -742,16 +748,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -762,16 +768,16 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
         <v>4</v>
@@ -782,19 +788,19 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -802,16 +808,16 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F6" t="s">
         <v>9</v>
@@ -819,42 +825,42 @@
     </row>
     <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -862,16 +868,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
@@ -882,16 +888,16 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -902,16 +908,16 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
         <v>9</v>
@@ -922,56 +928,56 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" t="s">
-        <v>14</v>
+        <v>24</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" t="s">
-        <v>17</v>
+        <v>72</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>73</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="F14" t="s">
         <v>9</v>
@@ -979,19 +985,19 @@
     </row>
     <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>9</v>
@@ -999,19 +1005,19 @@
     </row>
     <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F16" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Added registration error fields locators and bug report
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\Python\QA_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5738143-B461-46C0-9DC0-A38418DF91B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA3E36D-09AE-41AD-B3FC-9B2A63A4F7FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8FBF4EF6-23A4-453E-A09F-460DDE2B30EF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8FBF4EF6-23A4-453E-A09F-460DDE2B30EF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="Bug Report" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="85">
   <si>
     <t>ID</t>
   </si>
@@ -319,6 +320,41 @@
   </si>
   <si>
     <t>user can see empty cart</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Environment Details</t>
+  </si>
+  <si>
+    <t>Steps to Reproduce</t>
+  </si>
+  <si>
+    <t>Expected vs. Actual Result</t>
+  </si>
+  <si>
+    <t>Automation Artifacts</t>
+  </si>
+  <si>
+    <t>Registration Succeeds when the Password is more than 20 characters.</t>
+  </si>
+  <si>
+    <t>Environment: QA, Browser: Chrome, OS: Windows 11, Automation Tool: Robot Framework + SeleniumLibrary</t>
+  </si>
+  <si>
+    <t>1. Open browser
+2. Navigate to 'https://demo.opencartmart.com/ordercoupon/index.php?route=account/register'
+3. Populate registration fields with data: MyFirstName    MyLastName    testgmail@gmail.com    03535266242    MyVeryLongPassword200    MyVeryLongPassword200
+4. Click 'Accept Privacy Policy'
+5. Click 'Continue' button</t>
+  </si>
+  <si>
+    <t>Expected: User gets error under 'Password' field: Password must be between 4 and 20 characters!
+Actual:        User is registered successfully.</t>
+  </si>
+  <si>
+    <t>Error Screenshot, log.html</t>
   </si>
 </sst>
 </file>
@@ -694,16 +730,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A021F8-77F7-49B4-AF4C-68F5356311C2}">
   <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="3" width="52.140625" customWidth="1"/>
+    <col min="1" max="2" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="52.109375" customWidth="1"/>
     <col min="4" max="4" width="68" customWidth="1"/>
-    <col min="5" max="5" width="64.5703125" customWidth="1"/>
+    <col min="5" max="5" width="64.5546875" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -723,7 +759,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -743,7 +779,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -763,7 +799,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -783,7 +819,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -803,7 +839,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -823,7 +859,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>23</v>
       </c>
@@ -843,7 +879,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -863,7 +899,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -883,7 +919,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -903,7 +939,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -923,7 +959,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -943,7 +979,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -963,7 +999,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -983,7 +1019,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -1003,7 +1039,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -1021,6 +1057,60 @@
       </c>
       <c r="F16" t="s">
         <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FECD48BE-4DCD-4609-A045-C0DE0B1423EC}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48.77734375" customWidth="1"/>
+    <col min="2" max="2" width="90.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>